<commit_message>
Daily attendance processing - 2026-05-11 22:02:49 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y2_B2526_Respiratory_session_analysis.xlsx
+++ b/attendance_reports/Y2_B2526_Respiratory_session_analysis.xlsx
@@ -6013,7 +6013,7 @@
       </c>
       <c r="G112" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H112" s="5" t="inlineStr">
@@ -6737,7 +6737,7 @@
       </c>
       <c r="G128" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2024/2025</t>
+          <t>2024/2025, 2025/2026</t>
         </is>
       </c>
       <c r="H128" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-13 03:59:44 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y2_B2526_Respiratory_session_analysis.xlsx
+++ b/attendance_reports/Y2_B2526_Respiratory_session_analysis.xlsx
@@ -479,7 +479,7 @@
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="11" max="11"/>
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7">
@@ -846,7 +846,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8">
@@ -953,7 +953,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>47.7%</t>
+          <t>43.0%</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>57.5%</t>
+          <t>57.0%</t>
         </is>
       </c>
     </row>
@@ -1385,22 +1385,22 @@
         <v>16</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>43.8%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>66.3%</t>
+          <t>67.8%</t>
         </is>
       </c>
     </row>
@@ -1643,49 +1643,45 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>ANATOMY</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>13/11/2025</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>121/217</t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>0/217</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
@@ -1705,22 +1701,22 @@
         <v>16</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>43.8%</t>
         </is>
       </c>
       <c r="S20" s="4" t="inlineStr">
         <is>
-          <t>62.0%</t>
+          <t>58.9%</t>
         </is>
       </c>
     </row>
@@ -1783,22 +1779,22 @@
         <v>16</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q21" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R21" s="4" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="S21" s="4" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>55.1%</t>
         </is>
       </c>
     </row>
@@ -1865,22 +1861,22 @@
         <v>16</v>
       </c>
       <c r="O22" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P22" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R22" s="4" t="inlineStr">
         <is>
-          <t>56.2%</t>
+          <t>43.8%</t>
         </is>
       </c>
       <c r="S22" s="4" t="inlineStr">
         <is>
-          <t>37.7%</t>
+          <t>36.4%</t>
         </is>
       </c>
     </row>
@@ -4681,49 +4677,45 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="5" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="B84" s="5" t="inlineStr">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>B2</t>
         </is>
       </c>
-      <c r="C84" s="5" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>ANATOMY</t>
         </is>
       </c>
-      <c r="D84" s="5" t="inlineStr">
+      <c r="D84" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E84" s="5" t="inlineStr">
+      <c r="E84" s="2" t="inlineStr">
         <is>
           <t>13/11/2025</t>
         </is>
       </c>
-      <c r="F84" s="5" t="inlineStr">
+      <c r="F84" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="G84" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H84" s="5" t="inlineStr">
-        <is>
-          <t>187/224</t>
-        </is>
-      </c>
-      <c r="I84" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G84" s="2" t="inlineStr"/>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>0/224</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -5577,49 +5569,45 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="5" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="B104" s="5" t="inlineStr">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
         <is>
           <t>B3</t>
         </is>
       </c>
-      <c r="C104" s="5" t="inlineStr">
+      <c r="C104" s="2" t="inlineStr">
         <is>
           <t>MICROBIOLOGY</t>
         </is>
       </c>
-      <c r="D104" s="5" t="inlineStr">
+      <c r="D104" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E104" s="5" t="inlineStr">
+      <c r="E104" s="2" t="inlineStr">
         <is>
           <t>13/11/2025</t>
         </is>
       </c>
-      <c r="F104" s="5" t="inlineStr">
+      <c r="F104" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="G104" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H104" s="5" t="inlineStr">
-        <is>
-          <t>162/224</t>
-        </is>
-      </c>
-      <c r="I104" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G104" s="2" t="inlineStr"/>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>0/224</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -5945,49 +5933,45 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="5" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="B112" s="5" t="inlineStr">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
         <is>
           <t>B3</t>
         </is>
       </c>
-      <c r="C112" s="5" t="inlineStr">
+      <c r="C112" s="2" t="inlineStr">
         <is>
           <t>PHYSIOLOGY</t>
         </is>
       </c>
-      <c r="D112" s="5" t="inlineStr">
+      <c r="D112" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E112" s="5" t="inlineStr">
+      <c r="E112" s="2" t="inlineStr">
         <is>
           <t>13/11/2025</t>
         </is>
       </c>
-      <c r="F112" s="5" t="inlineStr">
+      <c r="F112" s="2" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G112" s="5" t="inlineStr">
-        <is>
-          <t>2024/2025, 2025/2026</t>
-        </is>
-      </c>
-      <c r="H112" s="5" t="inlineStr">
-        <is>
-          <t>172/224</t>
-        </is>
-      </c>
-      <c r="I112" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G112" s="2" t="inlineStr"/>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>0/224</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -6297,49 +6281,45 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="5" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="B120" s="5" t="inlineStr">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
         <is>
           <t>B4</t>
         </is>
       </c>
-      <c r="C120" s="5" t="inlineStr">
+      <c r="C120" s="2" t="inlineStr">
         <is>
           <t>MICROBIOLOGY</t>
         </is>
       </c>
-      <c r="D120" s="5" t="inlineStr">
+      <c r="D120" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E120" s="5" t="inlineStr">
+      <c r="E120" s="2" t="inlineStr">
         <is>
           <t>13/11/2025</t>
         </is>
       </c>
-      <c r="F120" s="5" t="inlineStr">
+      <c r="F120" s="2" t="inlineStr">
         <is>
           <t>10:00:00</t>
         </is>
       </c>
-      <c r="G120" s="5" t="inlineStr">
-        <is>
-          <t>2025/2026</t>
-        </is>
-      </c>
-      <c r="H120" s="5" t="inlineStr">
-        <is>
-          <t>117/226</t>
-        </is>
-      </c>
-      <c r="I120" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G120" s="2" t="inlineStr"/>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>0/226</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -6665,49 +6645,45 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="5" t="inlineStr">
-        <is>
-          <t>Year 2</t>
-        </is>
-      </c>
-      <c r="B128" s="5" t="inlineStr">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
         <is>
           <t>B4</t>
         </is>
       </c>
-      <c r="C128" s="5" t="inlineStr">
+      <c r="C128" s="2" t="inlineStr">
         <is>
           <t>PHYSIOLOGY</t>
         </is>
       </c>
-      <c r="D128" s="5" t="inlineStr">
+      <c r="D128" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E128" s="5" t="inlineStr">
+      <c r="E128" s="2" t="inlineStr">
         <is>
           <t>13/11/2025</t>
         </is>
       </c>
-      <c r="F128" s="5" t="inlineStr">
+      <c r="F128" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="G128" s="5" t="inlineStr">
-        <is>
-          <t>2024/2025, 2025/2026</t>
-        </is>
-      </c>
-      <c r="H128" s="5" t="inlineStr">
-        <is>
-          <t>73/226</t>
-        </is>
-      </c>
-      <c r="I128" s="5" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="G128" s="2" t="inlineStr"/>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>0/226</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>